<commit_message>
Raise Guangdong verified coverage to 37 (2.2x schools).
Merge expanded 2026 faculty/postdoc seeds and refresh validate/freshness/verify outputs for Guangdong.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/clean/economics/guangdong_listings_validated_2026-10-14.xlsx
+++ b/clean/economics/guangdong_listings_validated_2026-10-14.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -521,42 +521,42 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>广州</t>
+          <t>佛山</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Guangdong University of Finance and Economics</t>
+          <t>Foshan University</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>经济学院</t>
+          <t>经济贸易学院</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>“百万英才汇南粤”广东财经大学2026年博士后招聘公告</t>
+          <t>佛山大学数字经济【经济贸易学院-高层次人才】招聘</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>See announcement page</t>
+          <t>招满为止; 数字经济</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Dept/HR</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>http://rsc.gdufe.edu.cn/2026/0306/c4710a233784/page.htm</t>
+          <t>https://www.sciencehr.net/job/193240.html</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -573,37 +573,42 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Guangdong University of Finance and Economics</t>
+          <t>GDUF</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>大学人事处（含经济学博士后）</t>
+          <t>大数据与人工智能学院（金融统计）</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>广东财经大学2026年招聘博士后（经济学/管理学/法学等）</t>
+          <t>【百万英才汇南粤】广东金融学院2026年大数据与人工智能学院诚聘师资公告</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>常年诚聘; 含经济学</t>
+          <t>含金融统计与风险管理</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>http://rsc.gdufe.edu.cn/2026/0429/c4948a238378/page.htm</t>
+          <t>https://ai.gduf.edu.cn/info/1099/1240.htm</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>gdufrczp@gduf.edu.cn</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -620,7 +625,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Guangdong University of Finance and Economics</t>
+          <t>GDUT</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -630,27 +635,32 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>广东财经大学面向海内外招聘学科方向带头人的公告</t>
+          <t>广东工业大学经济学院优秀博士后招聘公告</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>See announcement page</t>
+          <t>jjrczhp@gdut.edu.cn</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Dept/HR</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>http://rsc.gdufe.edu.cn/2025/0116/c12800a215856/page.htm</t>
+          <t>https://jjxy.gdut.edu.cn/rczp/bsh.htm</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>jjrczhp@gdut.edu.cn</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -667,37 +677,42 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Guangdong University of Foreign Studies</t>
+          <t>GDUT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>人事处/人才招聘</t>
+          <t>经济学院</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>广东外语外贸大学2026年招聘师资博士后研究...</t>
+          <t>广东工业大学经济学院高层次人才招聘</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>See announcement page</t>
+          <t>青百计划教师岗</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Dept/HR</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>https://rsc.gdufs.edu.cn/info/1083/12549.htm</t>
+          <t>https://jjxy.gdut.edu.cn/info/1055/3235.htm</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>jjrczhp@gdut.edu.cn</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -714,37 +729,42 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Guangdong University of Foreign Studies</t>
+          <t>GDUT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>人事处/人才招聘</t>
+          <t>经济学院</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>广东外语外贸大学应用经济学博士后科研流动站2024年科研博士后研究人员招聘简章</t>
+          <t>百万英才汇南粤--广东工业大学高层次人才招聘简章（经济学院）</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>See announcement page</t>
+          <t>含经济学院博士后与青百</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Dept/HR</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>https://rsc.gdufs.edu.cn/info/1083/11977.htm</t>
+          <t>https://hr.gdut.edu.cn/info/1073/1195.htm</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>jjrczhp@gdut.edu.cn</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -761,17 +781,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Guangdong University of Foreign Studies</t>
+          <t>Guangdong University of Finance and Economics</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>人事处/人才招聘</t>
+          <t>经济学院</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>广东外语外贸大学应用经济学博士后科研流动站2025年科研博士后研究人员招聘简章</t>
+          <t>“百万英才汇南粤”广东财经大学2026年博士后招聘公告</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -786,7 +806,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>https://rsc.gdufs.edu.cn/info/1083/12041.htm</t>
+          <t>http://rsc.gdufe.edu.cn/2026/0306/c4710a233784/page.htm</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -808,32 +828,32 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Guangdong University of Foreign Studies</t>
+          <t>Guangdong University of Finance and Economics</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>人事处/人才招聘</t>
+          <t>大学人事处（含经济学博士后）</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>广东外语外贸大学应用经济学博士后科研流动站2026年科研博士后研究人员招聘简章</t>
+          <t>广东财经大学2026年招聘博士后（经济学/管理学/法学等）</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>See announcement page</t>
+          <t>常年诚聘; 含经济学</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Dept/HR</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>https://rsc.gdufs.edu.cn/info/1083/12519.htm</t>
+          <t>http://rsc.gdufe.edu.cn/2026/0429/c4948a238378/page.htm</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -855,37 +875,37 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Guangdong University of Foreign Studies</t>
+          <t>Guangdong University of Finance and Economics</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>人力资源部/经济贸易学院等</t>
+          <t>经济学院</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>广外2026年招聘师资博士后（含应用经济学、金融学）</t>
+          <t>广东财经大学面向海内外招聘学科方向带头人的公告</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>常年接受师资博士后申请</t>
+          <t>See announcement page</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>HR/学院</t>
+          <t>Dept/HR</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>https://rsc.gdufs.edu.cn/info/1017/12559.htm</t>
+          <t>http://rsc.gdufe.edu.cn/2025/0116/c12800a215856/page.htm</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -907,32 +927,32 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>经济贸易学院</t>
+          <t>人事处/人才招聘</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>广外2026年面向海内外招聘人才（经贸学院含国贸/产业/数字经济等）</t>
+          <t>广东外语外贸大学2026年招聘师资博士后研究...</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>见公告各学院联系人</t>
+          <t>See announcement page</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Email/学院</t>
+          <t>Dept/HR</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>https://rsc.gdufs.edu.cn/info/1017/12399.htm</t>
+          <t>https://rsc.gdufs.edu.cn/info/1083/12549.htm</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -954,32 +974,27 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>应用经济学博士后流动站</t>
+          <t>人事处/人才招聘</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>广外应用经济学博士后科研流动站2026年科研博士后招聘简章</t>
+          <t>广东外语外贸大学应用经济学博士后科研流动站2024年科研博士后研究人员招聘简章</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>gpszk@gdufs.edu.cn; 常年接受</t>
+          <t>See announcement page</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>HR/导师</t>
+          <t>Dept/HR</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>https://rsc.gdufs.edu.cn/info/1017/12909.htm</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>gpszk@gdufs.edu.cn</t>
+          <t>https://rsc.gdufs.edu.cn/info/1083/11977.htm</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1001,37 +1016,37 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Guangdong University of Technology</t>
+          <t>Guangdong University of Foreign Studies</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>经济学院</t>
+          <t>人事处/人才招聘</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>广东工业大学经济学院高层次人才招聘（应用经济学/数字经济/金融等）</t>
+          <t>广东外语外贸大学应用经济学博士后科研流动站2025年科研博士后研究人员招聘简章</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>简历发学院人才专员邮箱</t>
+          <t>See announcement page</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Dept/HR</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>https://jjxy.gdut.edu.cn/rczp/gccrc.htm</t>
+          <t>https://rsc.gdufs.edu.cn/info/1083/12041.htm</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -1048,32 +1063,32 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Guangzhou University</t>
+          <t>Guangdong University of Foreign Studies</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>经济与统计学院</t>
+          <t>人事处/人才招聘</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>广州大学经济与统计学院（李正辉课题组）2026年诚聘博士后</t>
+          <t>广东外语外贸大学应用经济学博士后科研流动站2026年科研博士后研究人员招聘简章</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>金融统计与风险管理、宏观经济统计等</t>
+          <t>See announcement page</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Dept/HR</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>https://www.gaoxiaojob.com/announcement/detail/388060.html</t>
+          <t>https://rsc.gdufs.edu.cn/info/1083/12519.htm</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1095,32 +1110,32 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Jinan University</t>
+          <t>Guangdong University of Foreign Studies</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>大学博士后流动站（含理论/应用经济学）</t>
+          <t>人力资源部/经济贸易学院等</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>暨南大学2026年博士后全球招聘（含应用经济学、理论经济学）</t>
+          <t>广外2026年招聘师资博士后（含应用经济学、金融学）</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>全年常态化接收</t>
+          <t>常年接受师资博士后申请</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>HR/导师</t>
+          <t>HR/学院</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>https://hrdam.jnu.edu.cn/2026/0413/c343a853500/page.htm</t>
+          <t>https://rsc.gdufs.edu.cn/info/1017/12559.htm</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1142,42 +1157,37 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Jinan University</t>
+          <t>Guangdong University of Foreign Studies</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>经济与社会研究院</t>
+          <t>经济贸易学院</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>暨南大学冯帅章教授团队招聘博士后</t>
+          <t>广外2026年面向海内外招聘人才（经贸学院含国贸/产业/数字经济等）</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>材料发 iesr@jnu.edu.cn</t>
+          <t>见公告各学院联系人</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Email/学院</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>https://iesr.jnu.edu.cn/2025/0624/c17209a839104/page.htm</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>iesr@jnu.edu.cn</t>
+          <t>https://rsc.gdufs.edu.cn/info/1017/12399.htm</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -1194,42 +1204,42 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Jinan University</t>
+          <t>Guangdong University of Foreign Studies</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>经济学院</t>
+          <t>应用经济学博士后流动站</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>暨南大学经济学院2025年诚聘海内外英才（含教师各层次与博士后）</t>
+          <t>广外应用经济学博士后科研流动站2026年科研博士后招聘简章</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>材料发 ojjy@jnu.edu.cn</t>
+          <t>gpszk@gdufs.edu.cn; 常年接受</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>HR/导师</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>https://ec.jnu.edu.cn/2024/1129/c42192a826585/page.htm</t>
+          <t>https://rsc.gdufs.edu.cn/info/1017/12909.htm</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>ojjy@jnu.edu.cn</t>
+          <t>gpszk@gdufs.edu.cn</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -1246,22 +1256,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>South China Normal University</t>
+          <t>Guangzhou University</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>经济与管理学院</t>
+          <t>经济与统计学院</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>华南师范大学经济与管理学院博士后流动站常年招收（理论/应用经济学）</t>
+          <t>广州大学2026年高层次人才招聘公告</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>scnujgzp@126.com; 常年招收</t>
+          <t>2026年度长期有效</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1271,17 +1281,12 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>http://em.scnu.edu.cn/xueshukeyan/boshihouliudongzhan/</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>scnujgzp@126.com</t>
+          <t>https://rsc.gzhu.edu.cn/info/1016/8191.htm</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -1298,32 +1303,32 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sun Yat-sen University</t>
+          <t>Guangzhou University</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>人事处/人才招聘</t>
+          <t>经济与统计学院</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2024-01-09 中山大学区域国别研究院面向海内外招聘博士后启事</t>
+          <t>广州大学经济与统计学院（李正辉课题组）2026年诚聘博士后</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>See announcement page</t>
+          <t>金融统计与风险管理、宏观经济统计等</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Dept/HR</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>https://rcb.sysu.edu.cn/article/532</t>
+          <t>https://www.gaoxiaojob.com/announcement/detail/388060.html</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1345,22 +1350,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Sun Yat-sen University</t>
+          <t>Guangzhou University</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>岭南学院/中观经济学研究院</t>
+          <t>经济与统计学院</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>中山大学中观经济学研究院公开招聘博士后</t>
+          <t>广州大学经济与统计学院（李正辉课题组）2026年诚聘博士后</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>长期有效; CV to sunyxi@mail.sysu.edu.cn</t>
+          <t>lizh@gzhu.edu.cn</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1370,12 +1375,12 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>https://lingnan.sysu.edu.cn/article/2774</t>
+          <t>https://www.gxszw.com/region/guangdong/gxzpgd/202603/30124547.html</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>sunyxi@mail.sysu.edu.cn</t>
+          <t>lizh@gzhu.edu.cn</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1392,27 +1397,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>珠海</t>
+          <t>广州</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sun Yat-sen University</t>
+          <t>Guangzhou University</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>国际金融学院</t>
+          <t>经济与统计学院</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>中山大学国际金融学院诚聘海内外英才（教师+博士后）</t>
+          <t>百万英才汇南粤 广州大学2026年博士后招聘简章</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>常年有效; 应用经济学等</t>
+          <t>常年有效; jjytjxy@163.com</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1422,12 +1427,17 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>https://isbf.sysu.edu.cn/zh-hans/article/2827</t>
+          <t>https://www.gzhu.edu.cn/info/1205/31377.htm</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>jjytjxy@163.com</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -1439,47 +1449,42 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>广州/深圳</t>
+          <t>广州</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sun Yat-sen University</t>
+          <t>Guangzhou University of Chinese Medicine</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>岭南学院</t>
+          <t>公共卫生与管理学院</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>中山大学岭南学院2026年招聘教师（含教研岗与博士后）</t>
+          <t>广州中医药大学2025-2026学年度学科博士后招收公告</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>CV to sunyxi@mail.sysu.edu.cn; rolling</t>
+          <t>全年接收进站申请</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>https://www.gaoxiaojob.com/announcement/detail/434822.html</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>sunyxi@mail.sysu.edu.cn</t>
+          <t>https://www.gzucm.edu.cn/info/1461/114061.htm</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -1491,42 +1496,1126 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Guangzhou University of Chinese Medicine</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>人事部（经济与管理类）</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>广州中医药大学诚聘海内外英才（含经济与管理类）</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>杏林学者; 经济与管理类</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>https://rsc.gzucm.edu.cn/info/1003/4003.htm</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Jinan University</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>经济与社会研究院</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Job Openings IESR 2026</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>iesr@jnu.edu.cn</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>AEA/Email</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>https://iesr.jnu.edu.cn/2025/1021/c17720a844641/page.htm</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>iesr@jnu.edu.cn</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Jinan University</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>经济学院</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>招聘通知｜暨南大学经济学院2025年诚聘海内外英才</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>ojjy@jnu.edu.cn</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>https://ec.jnu.edu.cn/2024/1129/c24919a826585/page.htm</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>ojjy@jnu.edu.cn</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Jinan University</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>大学博士后流动站（含理论/应用经济学）</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>暨南大学2026年博士后全球招聘公告</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>全年常态化接收</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>https://hrdam.jnu.edu.cn/2026/0413/c264a853500/page.htm</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Jinan University</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>大学博士后流动站（含理论/应用经济学）</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>暨南大学2026年博士后全球招聘（含应用经济学、理论经济学）</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>全年常态化接收</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>HR/导师</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>https://hrdam.jnu.edu.cn/2026/0413/c343a853500/page.htm</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Jinan University</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>经济与社会研究院</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>暨南大学冯帅章教授团队招聘博士后</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>材料发 iesr@jnu.edu.cn</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>https://iesr.jnu.edu.cn/2025/0624/c17209a839104/page.htm</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>iesr@jnu.edu.cn</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Jinan University</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>经济学院</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>暨南大学经济学院2025年诚聘海内外英才（含教师各层次与博士后）</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>材料发 ojjy@jnu.edu.cn</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>https://ec.jnu.edu.cn/2024/1129/c42192a826585/page.htm</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>ojjy@jnu.edu.cn</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>SCAU</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>经济管理学院</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>华南农业大学经济管理学院姜百臣教授研究团队招聘博士后启事</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>紫荆/全职博士后</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>https://cem.scau.edu.cn/2025/0221/c9875a399607/page.htm</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>SCAU</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>经济管理学院</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>华南农业大学经济管理学院易法敏教授研究团队招聘博士后</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>理论/应用经济学/数字经济/金融学</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>https://cem.scau.edu.cn/2025/0221/c9875a399618/page.htm</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>SCAU</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>经济管理学院</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>华南农业大学经济管理学院杨学儒教授研究团队招聘博士后启事</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>紫荆/全职博士后</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>https://cem.scau.edu.cn/2025/0221/c9875a399608/page.htm</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>SCAU</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>经济管理学院</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>华南农业大学经济管理学院柳松教授研究团队招聘博士后启事</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>紫荆/全职博士后</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>https://cem.scau.edu.cn/2025/0221/c9875a399594/page.htm</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>SCAU</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>经济管理学院</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>华南农业大学经济管理学院段伟教授研究团队招聘博士后启事</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>紫荆/全职博士后</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>https://cem.scau.edu.cn/2025/0221/c9875a399586/page.htm</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>SCNU</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>经济与管理学院</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>华南师范大学2025年公开招聘教学科研人员公告</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>见岗位表</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>http://em.scnu.edu.cn/a/20250910/10765.html</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>SCUT</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>经济与金融学院</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>华南理工大学经济与金融学院2025年招聘博士后公告</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>应用经济学; jjjrhr@scut.edu.cn</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gaoxiaojob.com/announcement/detail/305893.html</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>jjjrhr@scut.edu.cn</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>汕头</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Shantou University</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>商学院</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>汕头大学商学院博士后招聘（数字经济/宏观经济/产业经济）</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>全年接受入站申请</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>https://biz.stu.edu.cn/gk/cpyc/bshzp.htm</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>biz_recruitment@stu.edu.cn</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>汕头</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Shantou University</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>商学院</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>汕头大学商学院教师招聘（含应用经济学/数字经济）</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>biz_recruitment@stu.edu.cn</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Online/Email</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>https://biz.stu.edu.cn/gk/cpyc/jszp.htm</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>biz_recruitment@stu.edu.cn</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>South China Normal University</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>经济与管理学院</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>华南师范大学经济与管理学院博士后流动站常年招收（理论/应用经济学）</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>scnujgzp@126.com; 常年招收</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>http://em.scnu.edu.cn/xueshukeyan/boshihouliudongzhan/</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>scnujgzp@126.com</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Sun Yat-sen University</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>人事处/人才招聘</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>2024-01-09 中山大学区域国别研究院面向海内外招聘博士后启事</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>See announcement page</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Dept/HR</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>https://rcb.sysu.edu.cn/article/532</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sun Yat-sen University</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>岭南学院/中观经济学研究院</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>中山大学中观经济学研究院公开招聘博士后</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>长期有效; CV to sunyxi@mail.sysu.edu.cn</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>https://lingnan.sysu.edu.cn/article/2774</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>sunyxi@mail.sysu.edu.cn</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>珠海</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Sun Yat-sen University</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>国际金融学院</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>中山大学国际金融学院诚聘海内外英才（教师+博士后）</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>常年有效; 应用经济学等</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>https://isbf.sysu.edu.cn/zh-hans/article/2827</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>广州/深圳</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>Sun Yat-sen University</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>岭南学院</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>中山大学岭南学院2026年招聘教师（含教研岗与博士后）</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>CV to sunyxi@mail.sysu.edu.cn; rolling</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gaoxiaojob.com/announcement/detail/434822.html</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>sunyxi@mail.sysu.edu.cn</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>广州/深圳</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Sun Yat-sen University</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>岭南学院</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>加入岭南·成就卓越 | 中山大学岭南学院全球招聘（教师+博士后）</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>See announcement; rolling</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="I43" s="2" t="inlineStr">
         <is>
           <t>https://lingnan.sysu.edu.cn/article/2580</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>江门</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Wuyi University</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>经济管理学院</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>五邑大学经济管理学院2026年招聘人才</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>金融学/数字金融</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gaoxiaojob.com/announcement/detail/399560.html</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -1574,6 +2663,50 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>